<commit_message>
Move Status column data to Notes column
</commit_message>
<xml_diff>
--- a/cleaned_billing_by_service.xlsx
+++ b/cleaned_billing_by_service.xlsx
@@ -841,14 +841,9 @@
       <c r="H2" t="n">
         <v>0</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Paid 2026-02-28: 85</t>
+          <t>Paid 2026-02-28: 85 | Paid</t>
         </is>
       </c>
     </row>
@@ -933,14 +928,9 @@
       <c r="H4" t="n">
         <v>-40</v>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overpayment credit: $40.00, what he got goin on? </t>
+          <t>Overpayment credit: $40.00, what he got goin on?  | Paid</t>
         </is>
       </c>
     </row>
@@ -983,14 +973,9 @@
       <c r="H5" t="n">
         <v>0</v>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Paid 2026-02-28: 40</t>
+          <t>Paid 2026-02-28: 40 | Paid</t>
         </is>
       </c>
     </row>
@@ -1020,11 +1005,6 @@
           <t>25</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Not Paid</t>
-        </is>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
           <t>9125990226</t>
@@ -1032,7 +1012,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Cash Payer</t>
+          <t>Cash Payer | Not Paid</t>
         </is>
       </c>
     </row>
@@ -1294,14 +1274,14 @@
           <t>25</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>9125200166</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
         <is>
           <t>Ready</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>9125200166</t>
         </is>
       </c>
     </row>
@@ -1889,14 +1869,14 @@
           <t>50</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>9125990319</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
         <is>
           <t>Past Due</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>9125990319</t>
         </is>
       </c>
     </row>
@@ -2057,14 +2037,14 @@
           <t>25</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>9125205176</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
         <is>
           <t>PAID TILL MAY</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>9125205176</t>
         </is>
       </c>
     </row>
@@ -2094,14 +2074,14 @@
           <t>25</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>4076179781</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
         <is>
           <t>Past Due</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>4076179781</t>
         </is>
       </c>
     </row>
@@ -2259,14 +2239,14 @@
           <t>25</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>9124876000</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
         <is>
           <t>TM</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>9124876000</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2281,7 @@
           <t>25</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>Past Due</t>
         </is>
@@ -2432,14 +2412,14 @@
           <t>50</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2295635085</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
         <is>
           <t>Past Due</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>2295635085</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2506,7 @@
           <t>50</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>Past Due</t>
         </is>
@@ -2568,7 +2548,7 @@
           <t>895</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>TM</t>
         </is>
@@ -2610,14 +2590,14 @@
           <t>184</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2295635085</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
         <is>
           <t>TM</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>2295635085</t>
         </is>
       </c>
     </row>
@@ -2660,11 +2640,6 @@
       <c r="H47" t="n">
         <v>0</v>
       </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
       <c r="J47" t="inlineStr">
         <is>
           <t>9125017931</t>
@@ -2672,7 +2647,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Paid 2026-02-28: 85</t>
+          <t>Paid 2026-02-28: 85 | Paid</t>
         </is>
       </c>
     </row>
@@ -2702,11 +2677,6 @@
           <t>50</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>PAID</t>
-        </is>
-      </c>
       <c r="J48" t="inlineStr">
         <is>
           <t>9125200781</t>
@@ -2714,7 +2684,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Cash Payer</t>
+          <t>Cash Payer | PAID</t>
         </is>
       </c>
     </row>
@@ -2754,14 +2724,14 @@
           <t>975</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>12295614006</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
         <is>
           <t>TM</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>12295614006</t>
         </is>
       </c>
     </row>
@@ -2801,14 +2771,14 @@
           <t>831</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2035267181</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
         <is>
           <t>TM</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>2035267181</t>
         </is>
       </c>
     </row>
@@ -3215,14 +3185,14 @@
           <t>100</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>STARLINK</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>TM</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>STARLINK</t>
         </is>
       </c>
     </row>
@@ -3409,7 +3379,7 @@
           <t>Ria</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>LAST PAID 02/01</t>
         </is>
@@ -3562,7 +3532,7 @@
           <t>Corey Grady</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>LAST PAID 2/3</t>
         </is>
@@ -3589,14 +3559,14 @@
           <t>George Grant</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>9125205574</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>LAST PAID 2/9</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>9125205574</t>
         </is>
       </c>
     </row>
@@ -3626,14 +3596,14 @@
           <t>170</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>9125999003</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
         <is>
           <t>TELL HER TO RETURN MODEM</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>9125999003</t>
         </is>
       </c>
     </row>
@@ -3710,14 +3680,14 @@
           <t>85</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>9122767999‬</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
         <is>
           <t>Ready</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>9122767999‬</t>
         </is>
       </c>
     </row>
@@ -3784,7 +3754,7 @@
           <t>864</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>LAST PAID 02/06</t>
         </is>
@@ -3895,7 +3865,7 @@
           <t>Kirsty Thomas - Willacoochee</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>LAST PAID 02/13</t>
         </is>
@@ -4013,7 +3983,7 @@
           <t>170</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>Not Paid</t>
         </is>
@@ -4235,14 +4205,14 @@
           <t>941</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2295074503</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
         <is>
           <t>LAST PAID 02/01</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>2295074503</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4252,7 @@
           <t>528</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>LAST PAID 02/12</t>
         </is>
@@ -4309,14 +4279,14 @@
           <t>Austin Tanner/Michelle Tanner</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>3868551779</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
         <is>
           <t>LAST PAID 02/14</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>3868551779</t>
         </is>
       </c>
     </row>
@@ -4472,14 +4442,14 @@
           <t>85</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>9019303350</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
         <is>
           <t>LAST PAID 12/23</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>9019303350</t>
         </is>
       </c>
     </row>
@@ -4645,14 +4615,14 @@
           <t>67.86</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>9125209492</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
         <is>
           <t>PARTIAL APPR 2/25</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>9125209492</t>
         </is>
       </c>
     </row>
@@ -4697,14 +4667,14 @@
           <t>100</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>9125990441</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
         <is>
           <t>TM</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>9125990441</t>
         </is>
       </c>
     </row>
@@ -4749,14 +4719,14 @@
           <t>85</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>19402033533</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
         <is>
           <t>TM</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>19402033533</t>
         </is>
       </c>
     </row>
@@ -4791,7 +4761,7 @@
           <t>85</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>LAST PAID 2/22</t>
         </is>
@@ -4823,11 +4793,6 @@
           <t>85</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>TM</t>
-        </is>
-      </c>
       <c r="J41" t="inlineStr">
         <is>
           <t>9123092990</t>
@@ -4835,7 +4800,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Paycheck</t>
+          <t>Paycheck | TM</t>
         </is>
       </c>
     </row>
@@ -4880,14 +4845,14 @@
           <t>85</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>9125202750</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
         <is>
           <t>TM</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>9125202750</t>
         </is>
       </c>
     </row>
@@ -4927,14 +4892,14 @@
           <t>170</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>9123817201</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
         <is>
           <t>Ready</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>9123817201</t>
         </is>
       </c>
     </row>
@@ -4986,7 +4951,7 @@
           <t>85</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>LAST PAID 01/29</t>
         </is>
@@ -5033,14 +4998,14 @@
           <t>85</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2292697698</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
         <is>
           <t>TM</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>2292697698</t>
         </is>
       </c>
     </row>
@@ -5085,14 +5050,14 @@
           <t>170</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>8502426321</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
         <is>
           <t>TM</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>8502426321</t>
         </is>
       </c>
     </row>
@@ -5137,7 +5102,7 @@
           <t>255</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>Ready</t>
         </is>
@@ -5184,14 +5149,14 @@
           <t>85</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>9125333440</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
         <is>
           <t>TM</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>9125333440</t>
         </is>
       </c>
     </row>
@@ -5216,7 +5181,7 @@
           <t>she paid for 2mo $170 on 2/25</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t>TM</t>
         </is>
@@ -5572,14 +5537,14 @@
           <t>85</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>9122887142</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>LAST PAID 02/01</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>9122887142</t>
         </is>
       </c>
     </row>
@@ -5688,14 +5653,14 @@
           <t>April Manac</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2293751262</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>LAST PAID 2/07</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>2293751262</t>
         </is>
       </c>
     </row>
@@ -5735,14 +5700,14 @@
           <t>519</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>9125200595</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>LAST PAID 2/3</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>9125200595</t>
         </is>
       </c>
     </row>
@@ -5856,7 +5821,7 @@
           <t>DO NOT HAVE IT</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>LAST PAID 02/17</t>
         </is>
@@ -6029,14 +5994,14 @@
           <t>85</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2294158173</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
         <is>
           <t>TM</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>2294158173</t>
         </is>
       </c>
     </row>
@@ -6081,14 +6046,14 @@
           <t>85</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>9125209090</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
         <is>
           <t>GET NEW CARD</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>9125209090</t>
         </is>
       </c>
     </row>
@@ -6133,14 +6098,14 @@
           <t>85</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>9125208098</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
         <is>
           <t>TM</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>9125208098</t>
         </is>
       </c>
     </row>
@@ -6185,14 +6150,14 @@
           <t>85</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>9125999468</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
         <is>
           <t>LAST PAID 01/23</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>9125999468</t>
         </is>
       </c>
     </row>
@@ -6222,11 +6187,6 @@
           <t>85</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>LAST PAID 02/13</t>
-        </is>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
           <t>9125999381</t>
@@ -6234,7 +6194,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Cash Payer</t>
+          <t>Cash Payer | LAST PAID 02/13</t>
         </is>
       </c>
     </row>
@@ -6279,14 +6239,14 @@
           <t>85</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2296307778</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
         <is>
           <t>TM</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>2296307778</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add manual due date editing feature
</commit_message>
<xml_diff>
--- a/cleaned_billing_by_service.xlsx
+++ b/cleaned_billing_by_service.xlsx
@@ -647,7 +647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -718,6 +718,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Due Day</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -730,7 +735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -801,6 +806,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Due Day</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -846,6 +856,9 @@
           <t>Paid 2026-02-28: 85 | Paid</t>
         </is>
       </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -888,6 +901,9 @@
           <t>9124876597</t>
         </is>
       </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -933,6 +949,9 @@
           <t>Overpayment credit: $40.00, what he got goin on?  | Paid</t>
         </is>
       </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -978,6 +997,9 @@
           <t>Paid 2026-02-28: 40 | Paid</t>
         </is>
       </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1015,6 +1037,9 @@
           <t>Cash Payer | Not Paid</t>
         </is>
       </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1052,6 +1077,9 @@
           <t>227</t>
         </is>
       </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1089,6 +1117,9 @@
           <t>334</t>
         </is>
       </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1126,6 +1157,9 @@
           <t>516</t>
         </is>
       </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1163,6 +1197,9 @@
           <t>892</t>
         </is>
       </c>
+      <c r="L10" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1205,6 +1242,9 @@
           <t>12295398310</t>
         </is>
       </c>
+      <c r="L11" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1247,6 +1287,9 @@
           <t>12295398310</t>
         </is>
       </c>
+      <c r="L12" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1284,6 +1327,9 @@
           <t>Ready</t>
         </is>
       </c>
+      <c r="L13" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1326,6 +1372,9 @@
           <t>7274063859</t>
         </is>
       </c>
+      <c r="L14" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1368,6 +1417,9 @@
           <t>9125200384</t>
         </is>
       </c>
+      <c r="L15" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1395,6 +1447,9 @@
           <t>2294243621</t>
         </is>
       </c>
+      <c r="L16" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1422,6 +1477,9 @@
           <t>061205271 -0343001306 Barbara Bradford</t>
         </is>
       </c>
+      <c r="L17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1464,6 +1522,9 @@
           <t>19125208961</t>
         </is>
       </c>
+      <c r="L18" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1501,6 +1562,9 @@
           <t>148</t>
         </is>
       </c>
+      <c r="L19" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1543,6 +1607,9 @@
           <t>9124876120</t>
         </is>
       </c>
+      <c r="L20" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1585,6 +1652,9 @@
           <t>2292516694</t>
         </is>
       </c>
+      <c r="L21" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1622,6 +1692,9 @@
           <t>066</t>
         </is>
       </c>
+      <c r="L22" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1664,6 +1737,9 @@
           <t>2294748202</t>
         </is>
       </c>
+      <c r="L23" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1706,6 +1782,9 @@
           <t>9125201004</t>
         </is>
       </c>
+      <c r="L24" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1748,6 +1827,9 @@
           <t>2294154141</t>
         </is>
       </c>
+      <c r="L25" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1785,6 +1867,9 @@
           <t>5163203295</t>
         </is>
       </c>
+      <c r="L26" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1827,6 +1912,9 @@
           <t>9125990319</t>
         </is>
       </c>
+      <c r="L27" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1879,6 +1967,9 @@
           <t>Past Due</t>
         </is>
       </c>
+      <c r="L28" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1911,6 +2002,9 @@
           <t>Pay at Store</t>
         </is>
       </c>
+      <c r="L29" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1953,6 +2047,9 @@
           <t>4076179781</t>
         </is>
       </c>
+      <c r="L30" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1995,6 +2092,9 @@
           <t>9125990226</t>
         </is>
       </c>
+      <c r="L31" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2047,6 +2147,9 @@
           <t>PAID TILL MAY</t>
         </is>
       </c>
+      <c r="L32" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2084,6 +2187,9 @@
           <t>Past Due</t>
         </is>
       </c>
+      <c r="L33" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2111,6 +2217,9 @@
           <t>TRIAL</t>
         </is>
       </c>
+      <c r="L34" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2138,6 +2247,9 @@
           <t>TRIAL</t>
         </is>
       </c>
+      <c r="L35" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2160,6 +2272,9 @@
           <t>Jess UPS</t>
         </is>
       </c>
+      <c r="L36" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2197,6 +2312,9 @@
           <t>112</t>
         </is>
       </c>
+      <c r="L37" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2249,6 +2367,9 @@
           <t>TM</t>
         </is>
       </c>
+      <c r="L38" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2286,6 +2407,9 @@
           <t>Past Due</t>
         </is>
       </c>
+      <c r="L39" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2328,6 +2452,9 @@
           <t>9125201752</t>
         </is>
       </c>
+      <c r="L40" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2370,6 +2497,9 @@
           <t>9125992775</t>
         </is>
       </c>
+      <c r="L41" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2422,6 +2552,9 @@
           <t>Past Due</t>
         </is>
       </c>
+      <c r="L42" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2464,6 +2597,9 @@
           <t>14789522680</t>
         </is>
       </c>
+      <c r="L43" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2511,6 +2647,9 @@
           <t>Past Due</t>
         </is>
       </c>
+      <c r="L44" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2553,6 +2692,9 @@
           <t>TM</t>
         </is>
       </c>
+      <c r="L45" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2600,6 +2742,9 @@
           <t>TM</t>
         </is>
       </c>
+      <c r="L46" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2650,6 +2795,9 @@
           <t>Paid 2026-02-28: 85 | Paid</t>
         </is>
       </c>
+      <c r="L47" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2687,6 +2835,9 @@
           <t>Cash Payer | PAID</t>
         </is>
       </c>
+      <c r="L48" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2734,6 +2885,9 @@
           <t>TM</t>
         </is>
       </c>
+      <c r="L49" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2780,6 +2934,9 @@
         <is>
           <t>TM</t>
         </is>
+      </c>
+      <c r="L50" t="n">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -2793,7 +2950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2865,6 +3022,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Due Day</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2901,6 +3063,9 @@
         <is>
           <t>9125201247</t>
         </is>
+      </c>
+      <c r="L2" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -2914,7 +3079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2986,6 +3151,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Due Day</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3013,6 +3183,9 @@
           <t>Cash Payer</t>
         </is>
       </c>
+      <c r="L2" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3040,6 +3213,9 @@
           <t>Cash Payer</t>
         </is>
       </c>
+      <c r="L3" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3067,6 +3243,9 @@
           <t>Cash Payer</t>
         </is>
       </c>
+      <c r="L4" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3094,6 +3273,9 @@
           <t>Cash Payer</t>
         </is>
       </c>
+      <c r="L5" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3131,6 +3313,9 @@
           <t>STARLINK</t>
         </is>
       </c>
+      <c r="L6" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3153,6 +3338,9 @@
           <t>STARLINK</t>
         </is>
       </c>
+      <c r="L7" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3194,6 +3382,9 @@
         <is>
           <t>TM</t>
         </is>
+      </c>
+      <c r="L8" t="n">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -3207,7 +3398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3278,6 +3469,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Due Day</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3320,6 +3516,9 @@
           <t>9125922801</t>
         </is>
       </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3357,6 +3556,9 @@
           <t>753</t>
         </is>
       </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3384,6 +3586,9 @@
           <t>LAST PAID 02/01</t>
         </is>
       </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3426,6 +3631,9 @@
           <t>9125345121</t>
         </is>
       </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3468,6 +3676,9 @@
           <t>2088814559</t>
         </is>
       </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3510,6 +3721,9 @@
           <t>2705620807</t>
         </is>
       </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3537,6 +3751,9 @@
           <t>LAST PAID 2/3</t>
         </is>
       </c>
+      <c r="L8" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3569,6 +3786,9 @@
           <t>LAST PAID 2/9</t>
         </is>
       </c>
+      <c r="L9" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3606,6 +3826,9 @@
           <t>TELL HER TO RETURN MODEM</t>
         </is>
       </c>
+      <c r="L10" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3643,6 +3866,9 @@
           <t>504</t>
         </is>
       </c>
+      <c r="L11" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3690,6 +3916,9 @@
           <t>Ready</t>
         </is>
       </c>
+      <c r="L12" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3717,6 +3946,9 @@
           <t>9034139507</t>
         </is>
       </c>
+      <c r="L13" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3759,6 +3991,9 @@
           <t>LAST PAID 02/06</t>
         </is>
       </c>
+      <c r="L14" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3801,6 +4036,9 @@
           <t>9124875727</t>
         </is>
       </c>
+      <c r="L15" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3843,6 +4081,9 @@
           <t>12083203670</t>
         </is>
       </c>
+      <c r="L16" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3870,6 +4111,9 @@
           <t>LAST PAID 02/13</t>
         </is>
       </c>
+      <c r="L17" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3912,6 +4156,9 @@
           <t>9419620637</t>
         </is>
       </c>
+      <c r="L18" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3934,6 +4181,9 @@
           <t>AT WILLACOOCHEE</t>
         </is>
       </c>
+      <c r="L19" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3956,6 +4206,9 @@
           <t>AT WILLACOOCHEE</t>
         </is>
       </c>
+      <c r="L20" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3988,6 +4241,9 @@
           <t>Not Paid</t>
         </is>
       </c>
+      <c r="L21" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4015,6 +4271,9 @@
           <t>2295485050</t>
         </is>
       </c>
+      <c r="L22" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4042,6 +4301,9 @@
           <t>facebook</t>
         </is>
       </c>
+      <c r="L23" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4084,6 +4346,9 @@
           <t>2292697698</t>
         </is>
       </c>
+      <c r="L24" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4126,6 +4391,9 @@
           <t>9122811245</t>
         </is>
       </c>
+      <c r="L25" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4168,6 +4436,9 @@
           <t>9122887448</t>
         </is>
       </c>
+      <c r="L26" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4215,6 +4486,9 @@
           <t>LAST PAID 02/01</t>
         </is>
       </c>
+      <c r="L27" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4257,6 +4531,9 @@
           <t>LAST PAID 02/12</t>
         </is>
       </c>
+      <c r="L28" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4289,6 +4566,9 @@
           <t>LAST PAID 02/14</t>
         </is>
       </c>
+      <c r="L29" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4331,6 +4611,9 @@
           <t>9122866129</t>
         </is>
       </c>
+      <c r="L30" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4373,6 +4656,9 @@
           <t>9032598900</t>
         </is>
       </c>
+      <c r="L31" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4415,6 +4701,9 @@
           <t>9124878058</t>
         </is>
       </c>
+      <c r="L32" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4452,6 +4741,9 @@
           <t>LAST PAID 12/23</t>
         </is>
       </c>
+      <c r="L33" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4494,6 +4786,9 @@
           <t>7076317738</t>
         </is>
       </c>
+      <c r="L34" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4536,6 +4831,9 @@
           <t>9125345121</t>
         </is>
       </c>
+      <c r="L35" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4573,6 +4871,9 @@
           <t>944</t>
         </is>
       </c>
+      <c r="L36" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4625,6 +4926,9 @@
           <t>PARTIAL APPR 2/25</t>
         </is>
       </c>
+      <c r="L37" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4677,6 +4981,9 @@
           <t>TM</t>
         </is>
       </c>
+      <c r="L38" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4729,6 +5036,9 @@
           <t>TM</t>
         </is>
       </c>
+      <c r="L39" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4766,6 +5076,9 @@
           <t>LAST PAID 2/22</t>
         </is>
       </c>
+      <c r="L40" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4803,6 +5116,9 @@
           <t>Paycheck | TM</t>
         </is>
       </c>
+      <c r="L41" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4855,6 +5171,9 @@
           <t>TM</t>
         </is>
       </c>
+      <c r="L42" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4902,6 +5221,9 @@
           <t>Ready</t>
         </is>
       </c>
+      <c r="L43" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4924,6 +5246,9 @@
           <t>Cork Nashville</t>
         </is>
       </c>
+      <c r="L44" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4956,6 +5281,9 @@
           <t>LAST PAID 01/29</t>
         </is>
       </c>
+      <c r="L45" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5008,6 +5336,9 @@
           <t>TM</t>
         </is>
       </c>
+      <c r="L46" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5060,6 +5391,9 @@
           <t>TM</t>
         </is>
       </c>
+      <c r="L47" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5107,6 +5441,9 @@
           <t>Ready</t>
         </is>
       </c>
+      <c r="L48" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5159,6 +5496,9 @@
           <t>TM</t>
         </is>
       </c>
+      <c r="L49" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5186,6 +5526,9 @@
           <t>TM</t>
         </is>
       </c>
+      <c r="L50" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5208,6 +5551,9 @@
           <t>Ace Hardware</t>
         </is>
       </c>
+      <c r="L51" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5230,6 +5576,9 @@
           <t>Dockside</t>
         </is>
       </c>
+      <c r="L52" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5252,6 +5601,9 @@
           <t>Shop</t>
         </is>
       </c>
+      <c r="L53" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5274,6 +5626,9 @@
           <t>Tina Hendrix</t>
         </is>
       </c>
+      <c r="L54" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5295,6 +5650,9 @@
         <is>
           <t>Kayla Scott</t>
         </is>
+      </c>
+      <c r="L55" t="n">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -5308,7 +5666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5379,6 +5737,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Due Day</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5421,6 +5784,9 @@
           <t>9125201752</t>
         </is>
       </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5463,6 +5829,9 @@
           <t>STARLINK</t>
         </is>
       </c>
+      <c r="L3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5505,6 +5874,9 @@
           <t>19125926357</t>
         </is>
       </c>
+      <c r="L4" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5547,6 +5919,9 @@
           <t>LAST PAID 02/01</t>
         </is>
       </c>
+      <c r="L5" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5589,6 +5964,9 @@
           <t>2295607006</t>
         </is>
       </c>
+      <c r="L6" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5631,6 +6009,9 @@
           <t>9125200532</t>
         </is>
       </c>
+      <c r="L7" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5663,6 +6044,9 @@
           <t>LAST PAID 2/07</t>
         </is>
       </c>
+      <c r="L8" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5710,6 +6094,9 @@
           <t>LAST PAID 2/3</t>
         </is>
       </c>
+      <c r="L9" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5752,6 +6139,9 @@
           <t>9122825839</t>
         </is>
       </c>
+      <c r="L10" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5794,6 +6184,9 @@
           <t>4785504712</t>
         </is>
       </c>
+      <c r="L11" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5826,6 +6219,9 @@
           <t>LAST PAID 02/17</t>
         </is>
       </c>
+      <c r="L12" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5868,6 +6264,9 @@
           <t>9125990011</t>
         </is>
       </c>
+      <c r="L13" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5910,6 +6309,9 @@
           <t>9124709999</t>
         </is>
       </c>
+      <c r="L14" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5952,6 +6354,9 @@
           <t>7076317738</t>
         </is>
       </c>
+      <c r="L15" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6004,6 +6409,9 @@
           <t>TM</t>
         </is>
       </c>
+      <c r="L16" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6056,6 +6464,9 @@
           <t>GET NEW CARD</t>
         </is>
       </c>
+      <c r="L17" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6108,6 +6519,9 @@
           <t>TM</t>
         </is>
       </c>
+      <c r="L18" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6160,6 +6574,9 @@
           <t>LAST PAID 01/23</t>
         </is>
       </c>
+      <c r="L19" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6197,6 +6614,9 @@
           <t>Cash Payer | LAST PAID 02/13</t>
         </is>
       </c>
+      <c r="L20" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6248,6 +6668,9 @@
         <is>
           <t>TM</t>
         </is>
+      </c>
+      <c r="L21" t="n">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Notes2 column and editable field
</commit_message>
<xml_diff>
--- a/cleaned_billing_by_service.xlsx
+++ b/cleaned_billing_by_service.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="K-TV" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="MINT" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="STARLINK" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TMOB" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="VER1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K-TV" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MINT" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STARLINK" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMOB" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VER1" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -647,7 +647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -723,6 +723,11 @@
           <t>Due Day</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Notes2</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -735,7 +740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:M50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -811,6 +816,11 @@
           <t>Due Day</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Notes2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2950,7 +2960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3027,6 +3037,11 @@
           <t>Due Day</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Notes2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3079,7 +3094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3156,6 +3171,11 @@
           <t>Due Day</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Notes2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3398,7 +3418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:M55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3474,6 +3494,11 @@
           <t>Due Day</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Notes2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5666,7 +5691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5742,6 +5767,11 @@
           <t>Due Day</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Notes2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">

</xml_diff>

<commit_message>
Replace billing file with latest version
</commit_message>
<xml_diff>
--- a/cleaned_billing_by_service.xlsx
+++ b/cleaned_billing_by_service.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" tabRatio="600" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,13 @@
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -64,11 +71,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -740,23 +766,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M50"/>
+  <dimension ref="A1:M51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" style="7" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
     <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" style="9" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Charge Date</t>
         </is>
@@ -791,7 +817,7 @@
           <t>CVV</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>Amount Due</t>
         </is>
@@ -823,10 +849,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="A2" s="5" t="n">
+        <v>46113</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -858,23 +882,21 @@
           <t>253</t>
         </is>
       </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Paid 2026-02-28: 85 | Paid</t>
-        </is>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>2294748849</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="A3" s="5" t="n">
+        <v>46113</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -904,6 +926,11 @@
       <c r="G3" t="inlineStr">
         <is>
           <t>894</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -916,10 +943,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="A4" s="5" t="n">
+        <v>46113</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -951,23 +976,21 @@
           <t>759</t>
         </is>
       </c>
-      <c r="H4" t="n">
-        <v>-40</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Overpayment credit: $40.00, what he got goin on?  | Paid</t>
-        </is>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>2292928887</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="A5" s="6" t="n">
+        <v>46113</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -999,27 +1022,25 @@
           <t>826</t>
         </is>
       </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Paid 2026-02-28: 40 | Paid</t>
-        </is>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>9125508537</v>
       </c>
       <c r="L5" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="A6" s="5" t="n">
+        <v>46082</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>K-TV</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1032,7 +1053,7 @@
           <t>Charles Jones</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>25</t>
         </is>
@@ -1040,11 +1061,6 @@
       <c r="J6" t="inlineStr">
         <is>
           <t>9125990226</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Cash Payer | Not Paid</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -1052,10 +1068,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="A7" s="6" t="n">
+        <v>46113</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1086,16 +1100,22 @@
         <is>
           <t>227</t>
         </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>9125990553</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="A8" s="6" t="n">
+        <v>46113</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1125,6 +1145,11 @@
       <c r="G8" t="inlineStr">
         <is>
           <t>334</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -1132,10 +1157,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="A9" s="5" t="n">
+        <v>46114</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1149,33 +1172,39 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Matt Kenny Friend</t>
+          <t>Jared Jeffords</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>5146 2108 0044 7442</t>
+          <t>5148875080254847</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0427</t>
+          <t>0626</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>516</t>
-        </is>
+          <t>892</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>2295077932</v>
       </c>
       <c r="L9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-03-02</t>
-        </is>
+      <c r="A10" s="5" t="n">
+        <v>46114</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1189,22 +1218,32 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Jared Jeffords</t>
+          <t>Robin Casper</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>5148875080254847</t>
+          <t>5424181202361221</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0626</t>
+          <t>0727</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>892</t>
+          <t>012</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>12295398310</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1212,10 +1251,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-03-02</t>
-        </is>
+      <c r="A11" s="5" t="n">
+        <v>46114</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1229,7 +1266,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Robin Casper</t>
+          <t>Rachel Schools</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1245,6 +1282,11 @@
       <c r="G11" t="inlineStr">
         <is>
           <t>012</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1257,10 +1299,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-03-02</t>
-        </is>
+      <c r="A12" s="5" t="n">
+        <v>46083</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1274,27 +1314,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Rachel Schools</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>5424181202361221</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>0727</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>012</t>
+          <t>Rob Shirley</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>25</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>12295398310</t>
+          <t>9125200166</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1302,10 +1332,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-03-02</t>
-        </is>
+      <c r="A13" s="5" t="n">
+        <v>46114</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1319,22 +1347,32 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Rob Shirley</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>25</t>
+          <t>Blasé Kusterle</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>4147769462064441</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0928</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>072</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>9125200166</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Ready</t>
+          <t>7274063859</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1342,10 +1380,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-03-02</t>
-        </is>
+      <c r="A14" s="5" t="n">
+        <v>46114</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1359,27 +1395,32 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Blasé Kusterle</t>
+          <t>Rhett Barber</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>4147769462064441</t>
+          <t>5140680500425524</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0928</t>
+          <t>0128</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>072</t>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>7274063859</t>
+          <t>9125200384</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1387,10 +1428,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-03-02</t>
-        </is>
+      <c r="A15" s="5" t="n">
+        <v>46088</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1404,143 +1443,154 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Rhett Barber</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>5140680500425524</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
+          <t>Moses West</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2294243621</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>K-TV</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Talmadge Linda Friend</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>061205271 -0343001306 Barbara Bradford</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>2292928887</v>
+      </c>
+      <c r="L16" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>46119</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>K-TV</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Carlena Basonette</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>5538110009210839</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>1026</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>722</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>19125208961</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>46119</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>K-TV</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Kenny Corbitt</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>5140680500515225</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
         <is>
           <t>0128</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>006</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>9125200384</t>
-        </is>
-      </c>
-      <c r="L15" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>K-TV</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Moses West</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>2294243621</t>
-        </is>
-      </c>
-      <c r="L16" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>K-TV</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Talmadge Linda Friend</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>061205271 -0343001306 Barbara Bradford</t>
-        </is>
-      </c>
-      <c r="L17" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>K-TV</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Carlena Basonette</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>5538110009210839</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>1026</t>
-        </is>
-      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>722</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>19125208961</t>
-        </is>
+          <t>148</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>9125201009</v>
       </c>
       <c r="L18" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
+      <c r="A19" s="5" t="n">
+        <v>46119</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1549,27 +1599,37 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>45</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Kenny Corbitt</t>
+          <t>Albert Thornton</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>5140680500515225</t>
+          <t>5538110001919072</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0128</t>
+          <t>1126</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>9124876120</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -1577,10 +1637,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
+      <c r="A20" s="5" t="n">
+        <v>46119</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1589,32 +1647,37 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Albert Thornton</t>
+          <t>Louie Speedy Friend</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>5538110001919072</t>
+          <t>5178058002178096</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1126</t>
+          <t>0430</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>211</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>9124876120</t>
+          <t>2292516694</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -1622,14 +1685,12 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
+      <c r="A21" s="5" t="n">
+        <v>46119</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>K-TV</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1639,38 +1700,39 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Louie Speedy Friend</t>
+          <t>Brent James</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>5178058002178096</t>
+          <t>4159770018242239</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0430</t>
+          <t>0529</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>211</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>2292516694</t>
-        </is>
+          <t>066</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>9125200753</v>
       </c>
       <c r="L21" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
+      <c r="A22" s="5" t="n">
+        <v>46119</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1684,22 +1746,32 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Brent James</t>
+          <t>Otis Bailey</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>4159770018242239</t>
+          <t>4316800048077204</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0529</t>
+          <t>0726</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>066</t>
+          <t>738</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2294748202</t>
         </is>
       </c>
       <c r="L22" t="n">
@@ -1707,10 +1779,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
+      <c r="A23" s="5" t="n">
+        <v>46119</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1719,32 +1789,37 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>45</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Otis Bailey</t>
+          <t>Cecil Barber</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>4316800048077204</t>
+          <t>5140680500506679</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0726</t>
+          <t>1027</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>738</t>
+          <t>906</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2294748202</t>
+          <t>9125201004</t>
         </is>
       </c>
       <c r="L23" t="n">
@@ -1752,10 +1827,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
+      <c r="A24" s="5" t="n">
+        <v>46120</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1764,43 +1837,46 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Cecil Barber</t>
+          <t>Lynn Tucker</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>5140680500506679</t>
+          <t>5332480496672983</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>1027</t>
+          <t>0530</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>906</t>
+          <t>731</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>9125201004</t>
+          <t>2294154141</t>
         </is>
       </c>
       <c r="L24" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2026-03-08</t>
-        </is>
+      <c r="A25" s="5" t="n">
+        <v>46090</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1814,67 +1890,76 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Lynn Tucker</t>
+          <t>Alphanso Abner</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>5332480496672983</t>
+          <t>4147202566994388</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0530</t>
+          <t>0927</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>731</t>
-        </is>
+          <t>265</t>
+        </is>
+      </c>
+      <c r="H25" s="9" t="n">
+        <v>25</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2294154141</t>
+          <t>5163203295</t>
         </is>
       </c>
       <c r="L25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2026-03-09</t>
-        </is>
+      <c r="A26" s="5" t="n">
+        <v>46090</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
           <t>K-TV</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Alphanso Abner</t>
+          <t>Robert Seay</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>4147202566994388</t>
+          <t>5480281856411594</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0927</t>
+          <t>328</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>265</t>
-        </is>
+          <t>388</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>50</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>5163203295</t>
+          <t>9125990319</t>
         </is>
       </c>
       <c r="L26" t="n">
@@ -1882,10 +1967,8 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2026-03-09</t>
-        </is>
+      <c r="A27" s="5" t="n">
+        <v>46090</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1894,27 +1977,32 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Jacob Patton</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>5238910001896474</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>0528</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>890</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
           <t>50</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Robert Seay</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>5480281856411594</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>328</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>388</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1927,10 +2015,8 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2026-02-09</t>
-        </is>
+      <c r="A28" s="5" t="n">
+        <v>46090</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1944,37 +2030,15 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Jacob Patton</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>5238910001896474</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>0528</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>890</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
+          <t>Johnny Morgan</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>25</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
           <t>9125990319</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Past Due</t>
         </is>
       </c>
       <c r="L28" t="n">
@@ -1982,10 +2046,8 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2026-03-09</t>
-        </is>
+      <c r="A29" s="5" t="n">
+        <v>46090</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1999,17 +2061,30 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Johnny Morgan</t>
-        </is>
+          <t>Speedy Gonzales</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>5156768563049595</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>0230</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>607</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>25</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>9125990319</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>Pay at Store</t>
+          <t>4076179781</t>
         </is>
       </c>
       <c r="L29" t="n">
@@ -2017,10 +2092,8 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2026-03-09</t>
-        </is>
+      <c r="A30" s="5" t="n">
+        <v>46090</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2034,27 +2107,30 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Speedy Gonzales</t>
+          <t>Scott Lecessee</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>5156768563049595</t>
+          <t>5140680600752728</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>0230</t>
+          <t>01/29</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>607</t>
-        </is>
+          <t>626</t>
+        </is>
+      </c>
+      <c r="H30" s="9" t="n">
+        <v>25</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>4076179781</t>
+          <t>9125990226</t>
         </is>
       </c>
       <c r="L30" t="n">
@@ -2062,10 +2138,8 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>2026-03-09</t>
-        </is>
+      <c r="A31" s="5" t="n">
+        <v>46153</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2079,163 +2153,136 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Scott Lecessee</t>
+          <t>Chad Jones</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>5140680600752728</t>
+          <t>4190320032038857</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>01/29</t>
+          <t>1028</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>626</t>
+          <t>875</t>
+        </is>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>9125990226</t>
+          <t>9125205176</t>
         </is>
       </c>
       <c r="L31" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n">
+        <v>46062</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>K-TV</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Daryl Thomas</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>4076179781</t>
+        </is>
+      </c>
+      <c r="L32" t="n">
         <v>9</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>2026-05-11</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="5" t="n">
+        <v>46092</v>
+      </c>
+      <c r="B33" t="inlineStr">
         <is>
           <t>K-TV</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Chad Jones</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>4190320032038857</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>1028</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>875</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Miranda Odom</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>TRIAL</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>9125208688</v>
+      </c>
+      <c r="L33" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="n">
+        <v>46092</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>K-TV</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>9125205176</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>PAID TILL MAY</t>
-        </is>
-      </c>
-      <c r="L32" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>2026-02-09</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>K-TV</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Daryl Thomas</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>4076179781</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Past Due</t>
-        </is>
-      </c>
-      <c r="L33" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>K-TV</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Miranda Odom</t>
+          <t>Kirstin Soeder</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
           <t>TRIAL</t>
         </is>
+      </c>
+      <c r="J34" t="n">
+        <v>9125208605</v>
       </c>
       <c r="L34" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
+      <c r="A35" s="5" t="n">
+        <v>46092</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2249,23 +2296,19 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Kirstin Soeder</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>TRIAL</t>
-        </is>
+          <t>Jess UPS</t>
+        </is>
+      </c>
+      <c r="H35" s="9" t="n">
+        <v>25</v>
       </c>
       <c r="L35" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
+      <c r="A36" s="5" t="n">
+        <v>46094</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2279,18 +2322,37 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Jess UPS</t>
-        </is>
+          <t>Kimberly Tutt</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>4418379236341133</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>11/30</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
+      </c>
+      <c r="H36" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="J36" t="n">
+        <v>2294152632</v>
       </c>
       <c r="L36" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
+      <c r="A37" s="5" t="n">
+        <v>46098</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -2304,33 +2366,41 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Kimberly Tutt</t>
+          <t>David Harrel</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>4418379236341133</t>
+          <t>4305728842196305</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>11/30</t>
+          <t>0728</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>112</t>
+          <t>065</t>
+        </is>
+      </c>
+      <c r="H37" s="9" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>9124876000</t>
         </is>
       </c>
       <c r="L37" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
+      <c r="A38" s="5" t="n">
+        <v>46101</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -2344,48 +2414,33 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>David Harrel</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>4305728842196305</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>0728</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>065</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
+          <t>Danny Lecesse</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>5538110004597770</v>
+      </c>
+      <c r="F38" t="n">
+        <v>130</v>
+      </c>
+      <c r="G38" t="n">
+        <v>475</v>
+      </c>
+      <c r="H38" s="9" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>9124876000</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>TM</t>
-        </is>
+      <c r="J38" t="n">
+        <v>2293562355</v>
       </c>
       <c r="L38" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>2026-02-20</t>
-        </is>
+      <c r="A39" s="5" t="n">
+        <v>46101</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -2399,22 +2454,30 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Danny Lecesse</t>
+          <t>Jose Guadalupe</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>NEED NEW CARD THIS WAS EXPIRED</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>Past Due</t>
+          <t>5396890302394023</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>0830</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>236</t>
+        </is>
+      </c>
+      <c r="H39" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>9125201752</t>
         </is>
       </c>
       <c r="L39" t="n">
@@ -2422,10 +2485,8 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
+      <c r="A40" s="5" t="n">
+        <v>46101</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -2439,27 +2500,30 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Jose Guadalupe</t>
+          <t>Susan King</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>5396890302394023</t>
+          <t>5213331420581150</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>0830</t>
+          <t>1029</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>236</t>
-        </is>
+          <t>478</t>
+        </is>
+      </c>
+      <c r="H40" s="9" t="n">
+        <v>25</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>9125201752</t>
+          <t>9125992775</t>
         </is>
       </c>
       <c r="L40" t="n">
@@ -2467,10 +2531,8 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
+      <c r="A41" s="5" t="n">
+        <v>46074</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -2484,38 +2546,39 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Susan King</t>
+          <t>Lee Ricketson (Linda Friend)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>5213331420581150</t>
+          <t>4356190214839013</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>1029</t>
+          <t>0530</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>478</t>
-        </is>
+          <t>275</t>
+        </is>
+      </c>
+      <c r="H41" s="9" t="n">
+        <v>50</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>9125992775</t>
+          <t>2295635085</t>
         </is>
       </c>
       <c r="L41" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>2026-02-21</t>
-        </is>
+      <c r="A42" s="5" t="n">
+        <v>46103</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -2529,147 +2592,127 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Lee Ricketson (Linda Friend)</t>
+          <t>John Ried Linda Friend</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>4356190214839013</t>
+          <t>4400665620477636</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>0530</t>
+          <t>0528</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>275</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
+          <t>911</t>
+        </is>
+      </c>
+      <c r="H42" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>14789522680</t>
+        </is>
+      </c>
+      <c r="L42" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="n">
+        <v>46077</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>K-TV</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Doug Lowe</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>5121079824415407</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>0628</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>769</t>
+        </is>
+      </c>
+      <c r="H43" s="9" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>2295635085</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Past Due</t>
-        </is>
-      </c>
-      <c r="L42" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>2026-03-22</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
+      <c r="L43" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="n">
+        <v>46105</v>
+      </c>
+      <c r="B44" t="inlineStr">
         <is>
           <t>K-TV</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>John Ried Linda Friend</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>4400665620477636</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>0528</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>911</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>14789522680</t>
-        </is>
-      </c>
-      <c r="L43" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>2026-02-24</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>K-TV</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Doug Lowe</t>
+          <t>Charlie Kenny Jones</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>5121079824415407</t>
+          <t>4159770028121746</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>0628</t>
+          <t>0929</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>769</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Past Due</t>
-        </is>
+          <t>895</t>
+        </is>
+      </c>
+      <c r="H44" s="9" t="n">
+        <v>25</v>
       </c>
       <c r="L44" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>2026-03-24</t>
-        </is>
+      <c r="A45" s="5" t="n">
+        <v>46105</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>K-TV</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2679,27 +2722,30 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Charlie Kenny Jones</t>
+          <t>Emily Arnold</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>4159770028121746</t>
+          <t>5140680500470520</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>0929</t>
+          <t>0128</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>895</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>TM</t>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="H45" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2295635085</t>
         </is>
       </c>
       <c r="L45" t="n">
@@ -2707,10 +2753,8 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>2026-03-24</t>
-        </is>
+      <c r="A46" s="5" t="n">
+        <v>46105</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -2724,32 +2768,30 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Emily Arnold</t>
+          <t>Jacki Landrum</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>5140680500470520</t>
+          <t>5243001529691820</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>0128</t>
+          <t>1227</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>184</t>
-        </is>
+          <t>134</t>
+        </is>
+      </c>
+      <c r="H46" s="9" t="n">
+        <v>25</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2295635085</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>TM</t>
+          <t>9125017931</t>
         </is>
       </c>
       <c r="L46" t="n">
@@ -2757,10 +2799,8 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>2026-03-24</t>
-        </is>
+      <c r="A47" s="5" t="n">
+        <v>46105</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -2774,35 +2814,17 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Jacki Landrum</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>5243001529691820</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>1227</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>134</t>
-        </is>
-      </c>
-      <c r="H47" t="n">
-        <v>0</v>
+          <t>Timmy Manac</t>
+        </is>
+      </c>
+      <c r="H47" s="9" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>9125017931</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>Paid 2026-02-28: 85 | Paid</t>
+          <t>9125200781</t>
         </is>
       </c>
       <c r="L47" t="n">
@@ -2810,10 +2832,8 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>2026-03-24</t>
-        </is>
+      <c r="A48" s="5" t="n">
+        <v>46108</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -2827,33 +2847,39 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Timmy Manac</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
+          <t>Tara Linda Friend</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>5368099266210746</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>0229</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>975</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="n">
+        <v>25</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>9125200781</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>Cash Payer | PAID</t>
+          <t>12295614006</t>
         </is>
       </c>
       <c r="L48" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
+      <c r="A49" s="5" t="n">
+        <v>46108</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -2862,37 +2888,35 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>35</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Tara Linda Friend</t>
+          <t>Jaun Perez</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>5368099266210746</t>
+          <t>5108750028881829</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>0229</t>
+          <t>0528</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>975</t>
-        </is>
+          <t>831</t>
+        </is>
+      </c>
+      <c r="H49" s="9" t="n">
+        <v>35</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>12295614006</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>TM</t>
+          <t>2035267181</t>
         </is>
       </c>
       <c r="L49" t="n">
@@ -2900,10 +2924,8 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
+      <c r="A50" s="5" t="n">
+        <v>46166</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -2912,45 +2934,64 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Jaun Perez</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>5108750028881829</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>0528</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>831</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>2035267181</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>TM</t>
-        </is>
+          <t>Joanne Cribb</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>5218531601958560</v>
+      </c>
+      <c r="F50" t="n">
+        <v>328</v>
+      </c>
+      <c r="G50" t="n">
+        <v>559</v>
+      </c>
+      <c r="H50" s="9" t="n">
+        <v>25</v>
       </c>
       <c r="L50" t="n">
-        <v>27</v>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>K-TV</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Ben No Name</t>
+        </is>
+      </c>
+      <c r="H51" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>9125201142</v>
+      </c>
+      <c r="L51" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -3054,6 +3095,9 @@
           <t>MINT</t>
         </is>
       </c>
+      <c r="C2" t="n">
+        <v>85</v>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Haley Bass</t>
@@ -3073,6 +3117,9 @@
         <is>
           <t>741</t>
         </is>
+      </c>
+      <c r="H2" t="n">
+        <v>85</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -3188,10 +3235,16 @@
           <t>STARLINK</t>
         </is>
       </c>
+      <c r="C2" t="n">
+        <v>165</v>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Miranda Odom</t>
         </is>
+      </c>
+      <c r="H2" t="n">
+        <v>165</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -3278,10 +3331,16 @@
           <t>STARLINK</t>
         </is>
       </c>
+      <c r="C5" t="n">
+        <v>165</v>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>Kirstin Soeder</t>
         </is>
+      </c>
+      <c r="H5" t="n">
+        <v>165</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -3298,16 +3357,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-03-08</t>
-        </is>
+      <c r="A6" s="3" t="n">
+        <v>46120</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
           <t>STARLINK</t>
         </is>
       </c>
+      <c r="C6" t="n">
+        <v>175</v>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>Lily James</t>
@@ -3327,6 +3387,9 @@
         <is>
           <t>295</t>
         </is>
+      </c>
+      <c r="H6" t="n">
+        <v>175</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -3421,7 +3484,7 @@
   <dimension ref="A1:M55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" style="7" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="5"/>
@@ -3434,7 +3497,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Charge Date</t>
         </is>
@@ -3501,10 +3564,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="A2" s="5" t="n">
+        <v>46113</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -3534,6 +3595,11 @@
       <c r="G2" t="inlineStr">
         <is>
           <t>912</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -3546,10 +3612,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="A3" s="5" t="n">
+        <v>46113</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -3579,6 +3643,11 @@
       <c r="G3" t="inlineStr">
         <is>
           <t>753</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="L3" t="n">
@@ -3586,10 +3655,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="A4" s="5" t="n">
+        <v>46113</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -3606,9 +3673,9 @@
           <t>Ria</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>LAST PAID 02/01</t>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -3616,10 +3683,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="A5" s="5" t="n">
+        <v>46113</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -3649,6 +3714,11 @@
       <c r="G5" t="inlineStr">
         <is>
           <t>381</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -3661,10 +3731,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="A6" s="5" t="n">
+        <v>46113</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -3694,6 +3762,11 @@
       <c r="G6" t="inlineStr">
         <is>
           <t>527</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -3706,10 +3779,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="A7" s="5" t="n">
+        <v>46113</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -3739,6 +3810,11 @@
       <c r="G7" t="inlineStr">
         <is>
           <t>070</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -3751,7 +3827,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
@@ -3771,17 +3847,15 @@
           <t>Corey Grady</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>LAST PAID 2/3</t>
-        </is>
+      <c r="H8" t="n">
+        <v>85</v>
       </c>
       <c r="L8" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
@@ -3801,14 +3875,12 @@
           <t>George Grant</t>
         </is>
       </c>
+      <c r="H9" t="n">
+        <v>85</v>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>9125205574</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>LAST PAID 2/9</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -3816,7 +3888,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
@@ -3844,11 +3916,6 @@
       <c r="J10" t="inlineStr">
         <is>
           <t>9125999003</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>TELL HER TO RETURN MODEM</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -3856,10 +3923,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
+      <c r="A11" s="5" t="n">
+        <v>46117</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -3889,6 +3954,11 @@
       <c r="G11" t="inlineStr">
         <is>
           <t>504</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -3896,10 +3966,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
+      <c r="A12" s="5" t="n">
+        <v>46117</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -3928,17 +3996,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>85</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
           <t>9122767999‬</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Ready</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -3946,7 +4009,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>2026-03-06</t>
         </is>
@@ -3965,6 +4028,9 @@
         <is>
           <t xml:space="preserve">Kayla Scott Mom </t>
         </is>
+      </c>
+      <c r="H13" t="n">
+        <v>85</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -3976,7 +4042,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>2026-03-06</t>
         </is>
@@ -4011,20 +4077,16 @@
           <t>864</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>LAST PAID 02/06</t>
-        </is>
+      <c r="H14" t="n">
+        <v>85</v>
       </c>
       <c r="L14" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
+      <c r="A15" s="5" t="n">
+        <v>46119</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -4054,6 +4116,11 @@
       <c r="G15" t="inlineStr">
         <is>
           <t>572</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -4066,10 +4133,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
+      <c r="A16" s="5" t="n">
+        <v>46119</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -4099,6 +4164,11 @@
       <c r="G16" t="inlineStr">
         <is>
           <t>692</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -4111,7 +4181,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>2026-03-08</t>
         </is>
@@ -4131,17 +4201,15 @@
           <t>Kirsty Thomas - Willacoochee</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>LAST PAID 02/13</t>
-        </is>
+      <c r="H17" t="n">
+        <v>85</v>
       </c>
       <c r="L17" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>2026-03-09</t>
         </is>
@@ -4175,6 +4243,9 @@
         <is>
           <t>434</t>
         </is>
+      </c>
+      <c r="H18" t="n">
+        <v>85</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -4186,7 +4257,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>2026-03-09</t>
         </is>
@@ -4211,7 +4282,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>2026-03-09</t>
         </is>
@@ -4236,7 +4307,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>2026-03-09</t>
         </is>
@@ -4259,11 +4330,6 @@
       <c r="H21" t="inlineStr">
         <is>
           <t>170</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Not Paid</t>
         </is>
       </c>
       <c r="L21" t="n">
@@ -4271,7 +4337,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>2026-03-09</t>
         </is>
@@ -4301,7 +4367,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>2026-03-10</t>
         </is>
@@ -4320,6 +4386,9 @@
         <is>
           <t>Amanda Houston</t>
         </is>
+      </c>
+      <c r="H23" t="n">
+        <v>85</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -4331,7 +4400,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>2026-03-10</t>
         </is>
@@ -4365,6 +4434,9 @@
         <is>
           <t>379</t>
         </is>
+      </c>
+      <c r="H24" t="n">
+        <v>85</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -4376,7 +4448,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>
@@ -4410,6 +4482,9 @@
         <is>
           <t>808</t>
         </is>
+      </c>
+      <c r="H25" t="n">
+        <v>85</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -4421,7 +4496,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>
@@ -4455,6 +4530,9 @@
         <is>
           <t>220</t>
         </is>
+      </c>
+      <c r="H26" t="n">
+        <v>85</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -4466,7 +4544,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>
@@ -4501,14 +4579,12 @@
           <t>941</t>
         </is>
       </c>
+      <c r="H27" t="n">
+        <v>85</v>
+      </c>
       <c r="J27" t="inlineStr">
         <is>
           <t>2295074503</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>LAST PAID 02/01</t>
         </is>
       </c>
       <c r="L27" t="n">
@@ -4516,7 +4592,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>
@@ -4533,27 +4609,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Jesse Edwin Plumber</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>5140680500471825</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>1127</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>528</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>LAST PAID 02/12</t>
+          <t>ON HAND</t>
         </is>
       </c>
       <c r="L28" t="n">
@@ -4561,7 +4617,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
@@ -4581,14 +4637,12 @@
           <t>Austin Tanner/Michelle Tanner</t>
         </is>
       </c>
+      <c r="H29" t="n">
+        <v>85</v>
+      </c>
       <c r="J29" t="inlineStr">
         <is>
           <t>3868551779</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>LAST PAID 02/14</t>
         </is>
       </c>
       <c r="L29" t="n">
@@ -4596,7 +4650,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="7" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
@@ -4630,6 +4684,9 @@
         <is>
           <t>383</t>
         </is>
+      </c>
+      <c r="H30" t="n">
+        <v>85</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -4641,7 +4698,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>2026-03-14</t>
         </is>
@@ -4675,6 +4732,9 @@
         <is>
           <t>854</t>
         </is>
+      </c>
+      <c r="H31" t="n">
+        <v>85</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -4686,7 +4746,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>2026-03-16</t>
         </is>
@@ -4720,6 +4780,9 @@
         <is>
           <t>393</t>
         </is>
+      </c>
+      <c r="H32" t="n">
+        <v>85</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -4731,7 +4794,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>2026-02-17</t>
         </is>
@@ -4759,11 +4822,6 @@
       <c r="J33" t="inlineStr">
         <is>
           <t>9019303350</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>LAST PAID 12/23</t>
         </is>
       </c>
       <c r="L33" t="n">
@@ -4771,7 +4829,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
@@ -4805,6 +4863,9 @@
         <is>
           <t>161</t>
         </is>
+      </c>
+      <c r="H34" t="n">
+        <v>85</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
@@ -4816,10 +4877,8 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
+      <c r="A35" s="5" t="n">
+        <v>46130</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -4849,6 +4908,11 @@
       <c r="G35" t="inlineStr">
         <is>
           <t>901</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -4861,7 +4925,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="7" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -4895,13 +4959,16 @@
         <is>
           <t>944</t>
         </is>
+      </c>
+      <c r="H36" t="n">
+        <v>85</v>
       </c>
       <c r="L36" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>2026-02-20</t>
         </is>
@@ -4936,19 +5003,12 @@
           <t>065</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>67.86</t>
-        </is>
+      <c r="H37" t="n">
+        <v>85</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
           <t>9125209492</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>PARTIAL APPR 2/25</t>
         </is>
       </c>
       <c r="L37" t="n">
@@ -4956,7 +5016,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
@@ -4999,11 +5059,6 @@
       <c r="J38" t="inlineStr">
         <is>
           <t>9125990441</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>TM</t>
         </is>
       </c>
       <c r="L38" t="n">
@@ -5011,7 +5066,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
@@ -5054,11 +5109,6 @@
       <c r="J39" t="inlineStr">
         <is>
           <t>19402033533</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>TM</t>
         </is>
       </c>
       <c r="L39" t="n">
@@ -5066,7 +5116,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="7" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -5094,11 +5144,6 @@
       <c r="H40" t="inlineStr">
         <is>
           <t>85</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>LAST PAID 2/22</t>
         </is>
       </c>
       <c r="L40" t="n">
@@ -5106,7 +5151,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="7" t="inlineStr">
         <is>
           <t>2026-03-22</t>
         </is>
@@ -5134,11 +5179,6 @@
       <c r="J41" t="inlineStr">
         <is>
           <t>9123092990</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Paycheck | TM</t>
         </is>
       </c>
       <c r="L41" t="n">
@@ -5146,7 +5186,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="7" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
@@ -5189,11 +5229,6 @@
       <c r="J42" t="inlineStr">
         <is>
           <t>9125202750</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>TM</t>
         </is>
       </c>
       <c r="L42" t="n">
@@ -5201,10 +5236,8 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>2026-02-24</t>
-        </is>
+      <c r="A43" s="5" t="n">
+        <v>46105</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -5231,19 +5264,12 @@
           <t>0130</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>170</t>
-        </is>
+      <c r="H43" t="n">
+        <v>85</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
           <t>9123817201</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Ready</t>
         </is>
       </c>
       <c r="L43" t="n">
@@ -5251,7 +5277,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="7" t="inlineStr">
         <is>
           <t>2026-02-24</t>
         </is>
@@ -5276,10 +5302,8 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>2026-02-28</t>
-        </is>
+      <c r="A45" s="5" t="n">
+        <v>46109</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -5299,11 +5323,6 @@
       <c r="H45" t="inlineStr">
         <is>
           <t>85</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>LAST PAID 01/29</t>
         </is>
       </c>
       <c r="L45" t="n">
@@ -5311,7 +5330,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="7" t="inlineStr">
         <is>
           <t>2026-03-28</t>
         </is>
@@ -5354,11 +5373,6 @@
       <c r="J46" t="inlineStr">
         <is>
           <t>2292697698</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>TM</t>
         </is>
       </c>
       <c r="L46" t="n">
@@ -5366,7 +5380,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="7" t="inlineStr">
         <is>
           <t>2026-03-28</t>
         </is>
@@ -5401,19 +5415,12 @@
           <t>548</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>170</t>
-        </is>
+      <c r="H47" t="n">
+        <v>85</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
           <t>8502426321</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>TM</t>
         </is>
       </c>
       <c r="L47" t="n">
@@ -5421,7 +5428,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="7" t="inlineStr">
         <is>
           <t>2026-02-28</t>
         </is>
@@ -5456,22 +5463,15 @@
           <t>049</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
+      <c r="H48" t="n">
+        <v>340</v>
       </c>
       <c r="L48" t="n">
         <v>28</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="7" t="inlineStr">
         <is>
           <t>2026-03-28</t>
         </is>
@@ -5514,11 +5514,6 @@
       <c r="J49" t="inlineStr">
         <is>
           <t>9125333440</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>TM</t>
         </is>
       </c>
       <c r="L49" t="n">
@@ -5526,7 +5521,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="7" t="inlineStr">
         <is>
           <t>2026-04-18</t>
         </is>
@@ -5546,17 +5541,15 @@
           <t>she paid for 2mo $170 on 2/25</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>TM</t>
-        </is>
+      <c r="H50" t="n">
+        <v>-85</v>
       </c>
       <c r="L50" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="7" t="inlineStr">
         <is>
           <t>2026-01-24</t>
         </is>
@@ -5581,7 +5574,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="7" t="inlineStr">
         <is>
           <t>2026-01-24</t>
         </is>
@@ -5606,7 +5599,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="7" t="inlineStr">
         <is>
           <t>2026-02-05</t>
         </is>
@@ -5631,7 +5624,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="7" t="inlineStr">
         <is>
           <t>2026-01-30</t>
         </is>
@@ -5656,7 +5649,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="7" t="inlineStr">
         <is>
           <t>2026-01-11</t>
         </is>
@@ -5774,10 +5767,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="A2" s="3" t="n">
+        <v>46113</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -5808,6 +5799,9 @@
         <is>
           <t>236</t>
         </is>
+      </c>
+      <c r="H2" t="n">
+        <v>85</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -5819,10 +5813,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-03-02</t>
-        </is>
+      <c r="A3" s="3" t="n">
+        <v>46114</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -5853,6 +5845,9 @@
         <is>
           <t>422</t>
         </is>
+      </c>
+      <c r="H3" t="n">
+        <v>175</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -5864,10 +5859,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-03-04</t>
-        </is>
+      <c r="A4" s="3" t="n">
+        <v>46116</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -5898,6 +5891,9 @@
         <is>
           <t>973</t>
         </is>
+      </c>
+      <c r="H4" t="n">
+        <v>85</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -5909,10 +5905,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
-        </is>
+      <c r="A5" s="3" t="n">
+        <v>46118</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -5942,11 +5936,6 @@
       <c r="J5" t="inlineStr">
         <is>
           <t>9122887142</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>LAST PAID 02/01</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -5954,10 +5943,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
+      <c r="A6" s="3" t="n">
+        <v>46119</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -5988,6 +5975,9 @@
         <is>
           <t>506</t>
         </is>
+      </c>
+      <c r="H6" t="n">
+        <v>85</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -5999,10 +5989,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-03-08</t>
-        </is>
+      <c r="A7" s="3" t="n">
+        <v>46120</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -6033,6 +6021,9 @@
         <is>
           <t>484</t>
         </is>
+      </c>
+      <c r="H7" t="n">
+        <v>85</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -6064,14 +6055,12 @@
           <t>April Manac</t>
         </is>
       </c>
+      <c r="H8" t="n">
+        <v>85</v>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
           <t>2293751262</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>LAST PAID 2/07</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -6079,10 +6068,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-03-10</t>
-        </is>
+      <c r="A9" s="3" t="n">
+        <v>46122</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -6114,14 +6101,12 @@
           <t>519</t>
         </is>
       </c>
+      <c r="H9" t="n">
+        <v>85</v>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>9125200595</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>LAST PAID 2/3</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -6164,6 +6149,9 @@
           <t>502</t>
         </is>
       </c>
+      <c r="H10" t="n">
+        <v>85</v>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
           <t>9122825839</t>
@@ -6209,6 +6197,9 @@
           <t>436</t>
         </is>
       </c>
+      <c r="H11" t="n">
+        <v>85</v>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
           <t>4785504712</t>
@@ -6244,10 +6235,8 @@
           <t>DO NOT HAVE IT</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>LAST PAID 02/17</t>
-        </is>
+      <c r="H12" t="n">
+        <v>85</v>
       </c>
       <c r="L12" t="n">
         <v>13</v>
@@ -6289,6 +6278,9 @@
           <t>292</t>
         </is>
       </c>
+      <c r="H13" t="n">
+        <v>85</v>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
           <t>9125990011</t>
@@ -6334,6 +6326,9 @@
           <t>506</t>
         </is>
       </c>
+      <c r="H14" t="n">
+        <v>85</v>
+      </c>
       <c r="J14" t="inlineStr">
         <is>
           <t>9124709999</t>
@@ -6379,6 +6374,9 @@
           <t>161</t>
         </is>
       </c>
+      <c r="H15" t="n">
+        <v>85</v>
+      </c>
       <c r="J15" t="inlineStr">
         <is>
           <t>7076317738</t>
@@ -6434,11 +6432,6 @@
           <t>2294158173</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>TM</t>
-        </is>
-      </c>
       <c r="L16" t="n">
         <v>22</v>
       </c>
@@ -6479,19 +6472,12 @@
           <t>139</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>85</t>
-        </is>
+      <c r="H17" t="n">
+        <v>170</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
           <t>9125209090</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>GET NEW CARD</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -6544,20 +6530,13 @@
           <t>9125208098</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>TM</t>
-        </is>
-      </c>
       <c r="L18" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-02-23</t>
-        </is>
+      <c r="A19" s="3" t="n">
+        <v>46104</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -6597,11 +6576,6 @@
       <c r="J19" t="inlineStr">
         <is>
           <t>9125999468</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>LAST PAID 01/23</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -6639,11 +6613,6 @@
           <t>9125999381</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>Cash Payer | LAST PAID 02/13</t>
-        </is>
-      </c>
       <c r="L20" t="n">
         <v>27</v>
       </c>
@@ -6692,11 +6661,6 @@
       <c r="J21" t="inlineStr">
         <is>
           <t>2296307778</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>TM</t>
         </is>
       </c>
       <c r="L21" t="n">

</xml_diff>

<commit_message>
Add balance aging by month - shows current vs past due breakdown
</commit_message>
<xml_diff>
--- a/cleaned_billing_by_service.xlsx
+++ b/cleaned_billing_by_service.xlsx
@@ -673,7 +673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -754,6 +754,16 @@
           <t>Notes2</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Balance_History</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Balance_Current</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -766,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M51"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="7" min="1" max="1"/>
@@ -847,6 +857,16 @@
           <t>Notes2</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Balance_History</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Balance_Current</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
@@ -1066,6 +1086,9 @@
       <c r="L6" t="n">
         <v>1</v>
       </c>
+      <c r="O6" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
@@ -1330,6 +1353,9 @@
       <c r="L12" t="n">
         <v>2</v>
       </c>
+      <c r="O12" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
@@ -1457,6 +1483,9 @@
       <c r="L15" t="n">
         <v>7</v>
       </c>
+      <c r="O15" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
@@ -1919,6 +1948,9 @@
       <c r="L25" t="n">
         <v>9</v>
       </c>
+      <c r="O25" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n">
@@ -1965,6 +1997,9 @@
       <c r="L26" t="n">
         <v>9</v>
       </c>
+      <c r="O26" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
@@ -2013,6 +2048,9 @@
       <c r="L27" t="n">
         <v>9</v>
       </c>
+      <c r="O27" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n">
@@ -2044,6 +2082,9 @@
       <c r="L28" t="n">
         <v>9</v>
       </c>
+      <c r="O28" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n">
@@ -2090,6 +2131,9 @@
       <c r="L29" t="n">
         <v>9</v>
       </c>
+      <c r="O29" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n">
@@ -2136,6 +2180,9 @@
       <c r="L30" t="n">
         <v>9</v>
       </c>
+      <c r="O30" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n">
@@ -2217,6 +2264,9 @@
       <c r="L32" t="n">
         <v>9</v>
       </c>
+      <c r="O32" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n">
@@ -2305,6 +2355,9 @@
       <c r="L35" t="n">
         <v>11</v>
       </c>
+      <c r="O35" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n">
@@ -2349,6 +2402,9 @@
       <c r="L36" t="n">
         <v>13</v>
       </c>
+      <c r="O36" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n">
@@ -2397,6 +2453,9 @@
       <c r="L37" t="n">
         <v>17</v>
       </c>
+      <c r="O37" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
@@ -2437,6 +2496,9 @@
       <c r="L38" t="n">
         <v>20</v>
       </c>
+      <c r="O38" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n">
@@ -2483,6 +2545,9 @@
       <c r="L39" t="n">
         <v>20</v>
       </c>
+      <c r="O39" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n">
@@ -2529,6 +2594,9 @@
       <c r="L40" t="n">
         <v>20</v>
       </c>
+      <c r="O40" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n">
@@ -2575,6 +2643,9 @@
       <c r="L41" t="n">
         <v>21</v>
       </c>
+      <c r="O41" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n">
@@ -2621,6 +2692,9 @@
       <c r="L42" t="n">
         <v>22</v>
       </c>
+      <c r="O42" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n">
@@ -2664,6 +2738,9 @@
       <c r="L43" t="n">
         <v>24</v>
       </c>
+      <c r="O43" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n">
@@ -2705,6 +2782,9 @@
       <c r="L44" t="n">
         <v>24</v>
       </c>
+      <c r="O44" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n">
@@ -2751,6 +2831,9 @@
       <c r="L45" t="n">
         <v>24</v>
       </c>
+      <c r="O45" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n">
@@ -2797,6 +2880,9 @@
       <c r="L46" t="n">
         <v>24</v>
       </c>
+      <c r="O46" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n">
@@ -2830,6 +2916,9 @@
       <c r="L47" t="n">
         <v>24</v>
       </c>
+      <c r="O47" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n">
@@ -2876,6 +2965,9 @@
       <c r="L48" t="n">
         <v>27</v>
       </c>
+      <c r="O48" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n">
@@ -2922,6 +3014,9 @@
       <c r="L49" t="n">
         <v>27</v>
       </c>
+      <c r="O49" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n">
@@ -2956,6 +3051,9 @@
       </c>
       <c r="L50" t="n">
         <v>24</v>
+      </c>
+      <c r="O50" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="51">
@@ -3001,7 +3099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3083,6 +3181,16 @@
           <t>Notes2</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Balance_History</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Balance_Current</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3128,6 +3236,9 @@
       </c>
       <c r="L2" t="n">
         <v>9</v>
+      </c>
+      <c r="O2" t="n">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -3141,7 +3252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3223,6 +3334,16 @@
           <t>Notes2</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Balance_History</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Balance_Current</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3259,6 +3380,9 @@
       <c r="L2" t="n">
         <v>8</v>
       </c>
+      <c r="O2" t="n">
+        <v>165</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3354,6 +3478,9 @@
       </c>
       <c r="L5" t="n">
         <v>8</v>
+      </c>
+      <c r="O5" t="n">
+        <v>165</v>
       </c>
     </row>
     <row r="6">
@@ -3399,6 +3526,9 @@
       <c r="L6" t="n">
         <v>8</v>
       </c>
+      <c r="O6" t="n">
+        <v>175</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3468,6 +3598,9 @@
       </c>
       <c r="L8" t="n">
         <v>24</v>
+      </c>
+      <c r="O8" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -3481,7 +3614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M55"/>
+  <dimension ref="A1:O55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="7" min="1" max="1"/>
@@ -3562,6 +3695,16 @@
           <t>Notes2</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Balance_History</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Balance_Current</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
@@ -3853,6 +3996,9 @@
       <c r="L8" t="n">
         <v>3</v>
       </c>
+      <c r="O8" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -3886,6 +4032,9 @@
       <c r="L9" t="n">
         <v>3</v>
       </c>
+      <c r="O9" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -3920,6 +4069,9 @@
       </c>
       <c r="L10" t="n">
         <v>3</v>
+      </c>
+      <c r="O10" t="n">
+        <v>170</v>
       </c>
     </row>
     <row r="11">
@@ -4040,6 +4192,9 @@
       <c r="L13" t="n">
         <v>6</v>
       </c>
+      <c r="O13" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -4082,6 +4237,9 @@
       </c>
       <c r="L14" t="n">
         <v>6</v>
+      </c>
+      <c r="O14" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="15">
@@ -4207,6 +4365,9 @@
       <c r="L17" t="n">
         <v>8</v>
       </c>
+      <c r="O17" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -4255,6 +4416,9 @@
       <c r="L18" t="n">
         <v>9</v>
       </c>
+      <c r="O18" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -4335,6 +4499,9 @@
       <c r="L21" t="n">
         <v>9</v>
       </c>
+      <c r="O21" t="n">
+        <v>170</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -4398,6 +4565,9 @@
       <c r="L23" t="n">
         <v>10</v>
       </c>
+      <c r="O23" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -4446,6 +4616,9 @@
       <c r="L24" t="n">
         <v>10</v>
       </c>
+      <c r="O24" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -4494,6 +4667,9 @@
       <c r="L25" t="n">
         <v>11</v>
       </c>
+      <c r="O25" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -4542,6 +4718,9 @@
       <c r="L26" t="n">
         <v>11</v>
       </c>
+      <c r="O26" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -4590,6 +4769,9 @@
       <c r="L27" t="n">
         <v>11</v>
       </c>
+      <c r="O27" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -4648,6 +4830,9 @@
       <c r="L29" t="n">
         <v>13</v>
       </c>
+      <c r="O29" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -4696,6 +4881,9 @@
       <c r="L30" t="n">
         <v>13</v>
       </c>
+      <c r="O30" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -4744,6 +4932,9 @@
       <c r="L31" t="n">
         <v>14</v>
       </c>
+      <c r="O31" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -4792,6 +4983,9 @@
       <c r="L32" t="n">
         <v>16</v>
       </c>
+      <c r="O32" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -4827,6 +5021,9 @@
       <c r="L33" t="n">
         <v>17</v>
       </c>
+      <c r="O33" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -4874,6 +5071,9 @@
       </c>
       <c r="L34" t="n">
         <v>17</v>
+      </c>
+      <c r="O34" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="35">
@@ -4966,6 +5166,9 @@
       <c r="L36" t="n">
         <v>19</v>
       </c>
+      <c r="O36" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -5014,6 +5217,9 @@
       <c r="L37" t="n">
         <v>20</v>
       </c>
+      <c r="O37" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -5064,6 +5270,9 @@
       <c r="L38" t="n">
         <v>21</v>
       </c>
+      <c r="O38" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -5114,6 +5323,9 @@
       <c r="L39" t="n">
         <v>21</v>
       </c>
+      <c r="O39" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -5149,6 +5361,9 @@
       <c r="L40" t="n">
         <v>22</v>
       </c>
+      <c r="O40" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -5184,6 +5399,9 @@
       <c r="L41" t="n">
         <v>22</v>
       </c>
+      <c r="O41" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -5233,6 +5451,9 @@
       </c>
       <c r="L42" t="n">
         <v>23</v>
+      </c>
+      <c r="O42" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="43">
@@ -5275,6 +5496,9 @@
       <c r="L43" t="n">
         <v>24</v>
       </c>
+      <c r="O43" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -5328,6 +5552,9 @@
       <c r="L45" t="n">
         <v>28</v>
       </c>
+      <c r="O45" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -5378,6 +5605,9 @@
       <c r="L46" t="n">
         <v>28</v>
       </c>
+      <c r="O46" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -5426,6 +5656,9 @@
       <c r="L47" t="n">
         <v>28</v>
       </c>
+      <c r="O47" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -5469,6 +5702,9 @@
       <c r="L48" t="n">
         <v>28</v>
       </c>
+      <c r="O48" t="n">
+        <v>340</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -5519,6 +5755,9 @@
       <c r="L49" t="n">
         <v>28</v>
       </c>
+      <c r="O49" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -5546,6 +5785,9 @@
       </c>
       <c r="L50" t="n">
         <v>18</v>
+      </c>
+      <c r="O50" t="n">
+        <v>-85</v>
       </c>
     </row>
     <row r="51">
@@ -5684,7 +5926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5765,6 +6007,16 @@
           <t>Notes2</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Balance_History</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Balance_Current</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
@@ -5811,6 +6063,9 @@
       <c r="L2" t="n">
         <v>1</v>
       </c>
+      <c r="O2" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -5857,6 +6112,9 @@
       <c r="L3" t="n">
         <v>2</v>
       </c>
+      <c r="O3" t="n">
+        <v>175</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -5903,6 +6161,9 @@
       <c r="L4" t="n">
         <v>4</v>
       </c>
+      <c r="O4" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -5941,6 +6202,9 @@
       <c r="L5" t="n">
         <v>6</v>
       </c>
+      <c r="O5" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -5987,6 +6251,9 @@
       <c r="L6" t="n">
         <v>7</v>
       </c>
+      <c r="O6" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -6033,6 +6300,9 @@
       <c r="L7" t="n">
         <v>8</v>
       </c>
+      <c r="O7" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6065,6 +6335,9 @@
       </c>
       <c r="L8" t="n">
         <v>10</v>
+      </c>
+      <c r="O8" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="9">
@@ -6112,6 +6385,9 @@
       <c r="L9" t="n">
         <v>10</v>
       </c>
+      <c r="O9" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6160,6 +6436,9 @@
       <c r="L10" t="n">
         <v>10</v>
       </c>
+      <c r="O10" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6208,6 +6487,9 @@
       <c r="L11" t="n">
         <v>11</v>
       </c>
+      <c r="O11" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6241,6 +6523,9 @@
       <c r="L12" t="n">
         <v>13</v>
       </c>
+      <c r="O12" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6289,6 +6574,9 @@
       <c r="L13" t="n">
         <v>16</v>
       </c>
+      <c r="O13" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6337,6 +6625,9 @@
       <c r="L14" t="n">
         <v>17</v>
       </c>
+      <c r="O14" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6385,6 +6676,9 @@
       <c r="L15" t="n">
         <v>17</v>
       </c>
+      <c r="O15" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6435,6 +6729,9 @@
       <c r="L16" t="n">
         <v>22</v>
       </c>
+      <c r="O16" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6483,6 +6780,9 @@
       <c r="L17" t="n">
         <v>22</v>
       </c>
+      <c r="O17" t="n">
+        <v>170</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6532,6 +6832,9 @@
       </c>
       <c r="L18" t="n">
         <v>22</v>
+      </c>
+      <c r="O18" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="19">
@@ -6581,6 +6884,9 @@
       <c r="L19" t="n">
         <v>23</v>
       </c>
+      <c r="O19" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6616,6 +6922,9 @@
       <c r="L20" t="n">
         <v>27</v>
       </c>
+      <c r="O20" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6665,6 +6974,9 @@
       </c>
       <c r="L21" t="n">
         <v>28</v>
+      </c>
+      <c r="O21" t="n">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>